<commit_message>
new data for CAVV june 2026
</commit_message>
<xml_diff>
--- a/data/Prevencion_de_violencia_de_genero_CAVV/SAFEkits.xlsx
+++ b/data/Prevencion_de_violencia_de_genero_CAVV/SAFEkits.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gnper\Documents\ViolenciaGeneroPR\data\Prevencion_de_violencia_de_genero_CAVV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71727B3D-2C06-4B10-81E5-9599C7C230E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05399FCC-6F27-4939-915F-4263159D717E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="42">
   <si>
     <t>Equipo de recolección de evidencia en casos de violencia sexual (RAPE kits/ SAFE Kits)</t>
   </si>
@@ -172,7 +172,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -241,6 +241,17 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -274,7 +285,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="73">
+  <borders count="62">
     <border>
       <left/>
       <right/>
@@ -571,6 +582,293 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thick">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thick">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thick">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thick">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thick">
         <color rgb="FF000000"/>
       </left>
@@ -578,304 +876,6 @@
       <top style="thick">
         <color rgb="FF000000"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thick">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thick">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thick">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thick">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thick">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thick">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thick">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thick">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thick">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="thick">
-        <color rgb="FF000000"/>
-      </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -1067,149 +1067,13 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
+      <right/>
       <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thick">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thick">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1217,7 +1081,7 @@
         <color indexed="64"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </right>
       <top style="medium">
         <color indexed="64"/>
@@ -1228,8 +1092,8 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thick">
-        <color rgb="FF000000"/>
+      <left style="thin">
+        <color indexed="64"/>
       </left>
       <right style="medium">
         <color indexed="64"/>
@@ -1246,7 +1110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1323,10 +1187,16 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1335,7 +1205,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1344,16 +1214,13 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1365,10 +1232,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1377,20 +1247,11 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1398,13 +1259,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1419,26 +1280,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1446,19 +1292,13 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1470,56 +1310,21 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1566,62 +1371,68 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="10">
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
-        <left style="thick">
-          <color rgb="FF000000"/>
+        <left style="thin">
+          <color indexed="64"/>
         </left>
         <right style="thin">
-          <color rgb="FF000000"/>
+          <color indexed="64"/>
         </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="medium">
+          <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -1643,19 +1454,145 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
-          <color rgb="FF000000"/>
+          <color indexed="64"/>
         </left>
         <right style="thin">
-          <color rgb="FF000000"/>
+          <color indexed="64"/>
         </right>
         <top style="thin">
-          <color rgb="FF000000"/>
+          <color indexed="64"/>
         </top>
         <bottom style="thin">
-          <color rgb="FF000000"/>
+          <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -1687,92 +1624,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <border>
-        <bottom style="thick">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thick">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thick">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="medium">
           <color indexed="64"/>
         </top>
         <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thick">
           <color rgb="FF000000"/>
         </bottom>
       </border>
@@ -1791,8 +1647,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A48:B55" totalsRowShown="0" headerRowBorderDxfId="8" tableBorderDxfId="7">
-  <autoFilter ref="A48:B55" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A54:B63" totalsRowShown="0" headerRowBorderDxfId="4" tableBorderDxfId="9">
+  <autoFilter ref="A54:B63" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Año" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Total con querella" dataDxfId="5"/>
@@ -1802,11 +1658,11 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table2" displayName="Table2" ref="I48:J56" totalsRowShown="0" dataDxfId="3" headerRowBorderDxfId="4" tableBorderDxfId="2">
-  <autoFilter ref="I48:J56" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table2" displayName="Table2" ref="I54:J63" totalsRowShown="0" headerRowDxfId="0" dataDxfId="8" headerRowBorderDxfId="1" tableBorderDxfId="7">
+  <autoFilter ref="I54:J63" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Año" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Total sin querella" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Año" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Total sin querella" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2129,7 +1985,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M56"/>
+  <dimension ref="A1:M63"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" customWidth="1"/>
@@ -2142,37 +1998,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="98" t="s">
+      <c r="A1" s="79" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="98"/>
-      <c r="C1" s="98"/>
-      <c r="D1" s="98"/>
-      <c r="E1" s="98"/>
-      <c r="F1" s="98"/>
-      <c r="G1" s="98"/>
-      <c r="H1" s="98"/>
-      <c r="I1" s="98"/>
-      <c r="J1" s="98"/>
-      <c r="K1" s="98"/>
-      <c r="L1" s="98"/>
-      <c r="M1" s="98"/>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
+      <c r="E1" s="79"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="79"/>
+      <c r="I1" s="79"/>
+      <c r="J1" s="79"/>
+      <c r="K1" s="79"/>
+      <c r="L1" s="79"/>
+      <c r="M1" s="79"/>
     </row>
     <row r="3" spans="1:13" ht="21" x14ac:dyDescent="0.4">
-      <c r="A3" s="99" t="s">
+      <c r="A3" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="99"/>
-      <c r="C3" s="99"/>
-      <c r="D3" s="99"/>
-      <c r="E3" s="99"/>
-      <c r="I3" s="99" t="s">
+      <c r="B3" s="80"/>
+      <c r="C3" s="80"/>
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="I3" s="80" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="99"/>
-      <c r="K3" s="99"/>
-      <c r="L3" s="99"/>
-      <c r="M3" s="99"/>
+      <c r="J3" s="80"/>
+      <c r="K3" s="80"/>
+      <c r="L3" s="80"/>
+      <c r="M3" s="80"/>
     </row>
     <row r="4" spans="1:13" ht="31.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="24" t="s">
@@ -2207,7 +2063,7 @@
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="107">
+      <c r="A5" s="88">
         <v>2019</v>
       </c>
       <c r="B5" s="3" t="s">
@@ -2222,7 +2078,7 @@
       <c r="E5" s="3">
         <v>14</v>
       </c>
-      <c r="I5" s="110">
+      <c r="I5" s="70">
         <v>2019</v>
       </c>
       <c r="J5" s="3" t="s">
@@ -2234,12 +2090,12 @@
       <c r="L5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="M5" s="65">
+      <c r="M5" s="57">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="108"/>
+      <c r="A6" s="89"/>
       <c r="B6" s="7" t="s">
         <v>8</v>
       </c>
@@ -2252,7 +2108,7 @@
       <c r="E6" s="7">
         <v>13</v>
       </c>
-      <c r="I6" s="111"/>
+      <c r="I6" s="71"/>
       <c r="J6" s="7" t="s">
         <v>8</v>
       </c>
@@ -2262,12 +2118,12 @@
       <c r="L6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="M6" s="66">
+      <c r="M6" s="58">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="108"/>
+      <c r="A7" s="89"/>
       <c r="B7" s="5" t="s">
         <v>10</v>
       </c>
@@ -2280,7 +2136,7 @@
       <c r="E7" s="5">
         <v>10</v>
       </c>
-      <c r="I7" s="111"/>
+      <c r="I7" s="71"/>
       <c r="J7" s="5" t="s">
         <v>10</v>
       </c>
@@ -2290,12 +2146,12 @@
       <c r="L7" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="M7" s="67">
+      <c r="M7" s="59">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="108"/>
+      <c r="A8" s="89"/>
       <c r="B8" s="7" t="s">
         <v>12</v>
       </c>
@@ -2308,7 +2164,7 @@
       <c r="E8" s="7">
         <v>9</v>
       </c>
-      <c r="I8" s="111"/>
+      <c r="I8" s="71"/>
       <c r="J8" s="7" t="s">
         <v>12</v>
       </c>
@@ -2318,12 +2174,12 @@
       <c r="L8" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="M8" s="66">
+      <c r="M8" s="58">
         <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="108"/>
+      <c r="A9" s="89"/>
       <c r="B9" s="5" t="s">
         <v>14</v>
       </c>
@@ -2336,7 +2192,7 @@
       <c r="E9" s="5">
         <v>11</v>
       </c>
-      <c r="I9" s="111"/>
+      <c r="I9" s="71"/>
       <c r="J9" s="5" t="s">
         <v>14</v>
       </c>
@@ -2346,12 +2202,12 @@
       <c r="L9" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="M9" s="67">
+      <c r="M9" s="59">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="109"/>
+      <c r="A10" s="90"/>
       <c r="B10" s="10" t="s">
         <v>16</v>
       </c>
@@ -2364,7 +2220,7 @@
       <c r="E10" s="10">
         <v>14</v>
       </c>
-      <c r="I10" s="112"/>
+      <c r="I10" s="72"/>
       <c r="J10" s="10" t="s">
         <v>16</v>
       </c>
@@ -2374,12 +2230,12 @@
       <c r="L10" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="M10" s="68">
+      <c r="M10" s="60">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="107">
+      <c r="A11" s="88">
         <v>2020</v>
       </c>
       <c r="B11" s="3" t="s">
@@ -2394,24 +2250,24 @@
       <c r="E11" s="3">
         <v>5</v>
       </c>
-      <c r="I11" s="110">
+      <c r="I11" s="70">
         <v>2020</v>
       </c>
-      <c r="J11" s="69" t="s">
+      <c r="J11" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="K11" s="70">
+      <c r="K11" s="62">
         <v>2</v>
       </c>
-      <c r="L11" s="70" t="s">
+      <c r="L11" s="62" t="s">
         <v>7</v>
       </c>
-      <c r="M11" s="71">
+      <c r="M11" s="63">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="108"/>
+      <c r="A12" s="89"/>
       <c r="B12" s="7" t="s">
         <v>8</v>
       </c>
@@ -2424,7 +2280,7 @@
       <c r="E12" s="7">
         <v>13</v>
       </c>
-      <c r="I12" s="111"/>
+      <c r="I12" s="71"/>
       <c r="J12" s="7" t="s">
         <v>8</v>
       </c>
@@ -2434,12 +2290,12 @@
       <c r="L12" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="M12" s="66">
+      <c r="M12" s="58">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="108"/>
+      <c r="A13" s="89"/>
       <c r="B13" s="5" t="s">
         <v>10</v>
       </c>
@@ -2452,7 +2308,7 @@
       <c r="E13" s="5">
         <v>14</v>
       </c>
-      <c r="I13" s="111"/>
+      <c r="I13" s="71"/>
       <c r="J13" s="5" t="s">
         <v>10</v>
       </c>
@@ -2462,12 +2318,12 @@
       <c r="L13" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="M13" s="67">
+      <c r="M13" s="59">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="108"/>
+      <c r="A14" s="89"/>
       <c r="B14" s="7" t="s">
         <v>12</v>
       </c>
@@ -2480,7 +2336,7 @@
       <c r="E14" s="7">
         <v>19</v>
       </c>
-      <c r="I14" s="111"/>
+      <c r="I14" s="71"/>
       <c r="J14" s="7" t="s">
         <v>12</v>
       </c>
@@ -2490,12 +2346,12 @@
       <c r="L14" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="M14" s="66">
+      <c r="M14" s="58">
         <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="108"/>
+      <c r="A15" s="89"/>
       <c r="B15" s="5" t="s">
         <v>14</v>
       </c>
@@ -2508,7 +2364,7 @@
       <c r="E15" s="5">
         <v>9</v>
       </c>
-      <c r="I15" s="111"/>
+      <c r="I15" s="71"/>
       <c r="J15" s="5" t="s">
         <v>14</v>
       </c>
@@ -2518,12 +2374,12 @@
       <c r="L15" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="M15" s="67">
+      <c r="M15" s="59">
         <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="109"/>
+      <c r="A16" s="90"/>
       <c r="B16" s="10" t="s">
         <v>16</v>
       </c>
@@ -2536,7 +2392,7 @@
       <c r="E16" s="10">
         <v>9</v>
       </c>
-      <c r="I16" s="112"/>
+      <c r="I16" s="72"/>
       <c r="J16" s="10" t="s">
         <v>16</v>
       </c>
@@ -2546,12 +2402,12 @@
       <c r="L16" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="M16" s="68">
+      <c r="M16" s="60">
         <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="105">
+      <c r="A17" s="86">
         <v>2021</v>
       </c>
       <c r="B17" s="3" t="s">
@@ -2566,7 +2422,7 @@
       <c r="E17" s="42">
         <v>15</v>
       </c>
-      <c r="I17" s="101">
+      <c r="I17" s="82">
         <v>2021</v>
       </c>
       <c r="J17" s="3" t="s">
@@ -2583,7 +2439,7 @@
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A18" s="102"/>
+      <c r="A18" s="83"/>
       <c r="B18" s="7" t="s">
         <v>8</v>
       </c>
@@ -2596,7 +2452,7 @@
       <c r="E18" s="43">
         <v>13</v>
       </c>
-      <c r="I18" s="96"/>
+      <c r="I18" s="77"/>
       <c r="J18" s="7" t="s">
         <v>8</v>
       </c>
@@ -2611,7 +2467,7 @@
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A19" s="102"/>
+      <c r="A19" s="83"/>
       <c r="B19" s="5" t="s">
         <v>10</v>
       </c>
@@ -2624,7 +2480,7 @@
       <c r="E19" s="44">
         <v>7</v>
       </c>
-      <c r="I19" s="96"/>
+      <c r="I19" s="77"/>
       <c r="J19" s="5" t="s">
         <v>10</v>
       </c>
@@ -2639,7 +2495,7 @@
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A20" s="102"/>
+      <c r="A20" s="83"/>
       <c r="B20" s="7" t="s">
         <v>12</v>
       </c>
@@ -2652,7 +2508,7 @@
       <c r="E20" s="43">
         <v>9</v>
       </c>
-      <c r="I20" s="96"/>
+      <c r="I20" s="77"/>
       <c r="J20" s="7" t="s">
         <v>12</v>
       </c>
@@ -2667,7 +2523,7 @@
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A21" s="102"/>
+      <c r="A21" s="83"/>
       <c r="B21" s="5" t="s">
         <v>14</v>
       </c>
@@ -2680,7 +2536,7 @@
       <c r="E21" s="44">
         <v>10</v>
       </c>
-      <c r="I21" s="96"/>
+      <c r="I21" s="77"/>
       <c r="J21" s="5" t="s">
         <v>14</v>
       </c>
@@ -2695,7 +2551,7 @@
       </c>
     </row>
     <row r="22" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="106"/>
+      <c r="A22" s="87"/>
       <c r="B22" s="10" t="s">
         <v>16</v>
       </c>
@@ -2708,7 +2564,7 @@
       <c r="E22" s="45">
         <v>8</v>
       </c>
-      <c r="I22" s="100"/>
+      <c r="I22" s="81"/>
       <c r="J22" s="10" t="s">
         <v>16</v>
       </c>
@@ -2723,7 +2579,7 @@
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A23" s="104">
+      <c r="A23" s="85">
         <v>2022</v>
       </c>
       <c r="B23" s="3" t="s">
@@ -2738,7 +2594,7 @@
       <c r="E23" s="42">
         <v>7</v>
       </c>
-      <c r="I23" s="95">
+      <c r="I23" s="76">
         <v>2022</v>
       </c>
       <c r="J23" s="3" t="s">
@@ -2755,7 +2611,7 @@
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A24" s="102"/>
+      <c r="A24" s="83"/>
       <c r="B24" s="7" t="s">
         <v>8</v>
       </c>
@@ -2768,7 +2624,7 @@
       <c r="E24" s="43">
         <v>17</v>
       </c>
-      <c r="I24" s="96"/>
+      <c r="I24" s="77"/>
       <c r="J24" s="7" t="s">
         <v>8</v>
       </c>
@@ -2783,7 +2639,7 @@
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A25" s="102"/>
+      <c r="A25" s="83"/>
       <c r="B25" s="5" t="s">
         <v>10</v>
       </c>
@@ -2796,7 +2652,7 @@
       <c r="E25" s="44">
         <v>13</v>
       </c>
-      <c r="I25" s="96"/>
+      <c r="I25" s="77"/>
       <c r="J25" s="5" t="s">
         <v>10</v>
       </c>
@@ -2811,7 +2667,7 @@
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A26" s="102"/>
+      <c r="A26" s="83"/>
       <c r="B26" s="7" t="s">
         <v>12</v>
       </c>
@@ -2824,7 +2680,7 @@
       <c r="E26" s="43">
         <v>15</v>
       </c>
-      <c r="I26" s="96"/>
+      <c r="I26" s="77"/>
       <c r="J26" s="7" t="s">
         <v>12</v>
       </c>
@@ -2839,7 +2695,7 @@
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A27" s="102"/>
+      <c r="A27" s="83"/>
       <c r="B27" s="5" t="s">
         <v>14</v>
       </c>
@@ -2852,7 +2708,7 @@
       <c r="E27" s="44">
         <v>12</v>
       </c>
-      <c r="I27" s="96"/>
+      <c r="I27" s="77"/>
       <c r="J27" s="5" t="s">
         <v>14</v>
       </c>
@@ -2867,7 +2723,7 @@
       </c>
     </row>
     <row r="28" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="103"/>
+      <c r="A28" s="84"/>
       <c r="B28" s="10" t="s">
         <v>16</v>
       </c>
@@ -2880,7 +2736,7 @@
       <c r="E28" s="45">
         <v>20</v>
       </c>
-      <c r="I28" s="100"/>
+      <c r="I28" s="81"/>
       <c r="J28" s="10" t="s">
         <v>16</v>
       </c>
@@ -2895,7 +2751,7 @@
       </c>
     </row>
     <row r="29" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="102">
+      <c r="A29" s="83">
         <v>2023</v>
       </c>
       <c r="B29" s="3" t="s">
@@ -2910,7 +2766,7 @@
       <c r="E29" s="42">
         <v>9</v>
       </c>
-      <c r="I29" s="95">
+      <c r="I29" s="76">
         <v>2023</v>
       </c>
       <c r="J29" s="3" t="s">
@@ -2927,7 +2783,7 @@
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A30" s="102"/>
+      <c r="A30" s="83"/>
       <c r="B30" s="7" t="s">
         <v>8</v>
       </c>
@@ -2940,7 +2796,7 @@
       <c r="E30" s="43">
         <v>9</v>
       </c>
-      <c r="I30" s="96"/>
+      <c r="I30" s="77"/>
       <c r="J30" s="7" t="s">
         <v>8</v>
       </c>
@@ -2955,7 +2811,7 @@
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A31" s="102"/>
+      <c r="A31" s="83"/>
       <c r="B31" s="5" t="s">
         <v>10</v>
       </c>
@@ -2968,7 +2824,7 @@
       <c r="E31" s="44">
         <v>13</v>
       </c>
-      <c r="I31" s="96"/>
+      <c r="I31" s="77"/>
       <c r="J31" s="5" t="s">
         <v>10</v>
       </c>
@@ -2983,7 +2839,7 @@
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A32" s="102"/>
+      <c r="A32" s="83"/>
       <c r="B32" s="7" t="s">
         <v>12</v>
       </c>
@@ -2996,7 +2852,7 @@
       <c r="E32" s="43">
         <v>11</v>
       </c>
-      <c r="I32" s="96"/>
+      <c r="I32" s="77"/>
       <c r="J32" s="7" t="s">
         <v>12</v>
       </c>
@@ -3011,7 +2867,7 @@
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A33" s="102"/>
+      <c r="A33" s="83"/>
       <c r="B33" s="5" t="s">
         <v>14</v>
       </c>
@@ -3024,7 +2880,7 @@
       <c r="E33" s="44">
         <v>15</v>
       </c>
-      <c r="I33" s="96"/>
+      <c r="I33" s="77"/>
       <c r="J33" s="5" t="s">
         <v>14</v>
       </c>
@@ -3039,7 +2895,7 @@
       </c>
     </row>
     <row r="34" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="103"/>
+      <c r="A34" s="84"/>
       <c r="B34" s="18" t="s">
         <v>16</v>
       </c>
@@ -3052,7 +2908,7 @@
       <c r="E34" s="46">
         <v>11</v>
       </c>
-      <c r="I34" s="100"/>
+      <c r="I34" s="81"/>
       <c r="J34" s="18" t="s">
         <v>16</v>
       </c>
@@ -3067,7 +2923,7 @@
       </c>
     </row>
     <row r="35" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="92">
+      <c r="A35" s="73">
         <v>2024</v>
       </c>
       <c r="B35" s="40" t="s">
@@ -3082,7 +2938,7 @@
       <c r="E35" s="37">
         <v>20</v>
       </c>
-      <c r="I35" s="95">
+      <c r="I35" s="76">
         <v>2024</v>
       </c>
       <c r="J35" s="27" t="s">
@@ -3099,7 +2955,7 @@
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A36" s="93"/>
+      <c r="A36" s="74"/>
       <c r="B36" s="23" t="s">
         <v>8</v>
       </c>
@@ -3112,7 +2968,7 @@
       <c r="E36" s="38">
         <v>15</v>
       </c>
-      <c r="I36" s="96"/>
+      <c r="I36" s="77"/>
       <c r="J36" s="20" t="s">
         <v>8</v>
       </c>
@@ -3127,7 +2983,7 @@
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A37" s="93"/>
+      <c r="A37" s="74"/>
       <c r="B37" s="22" t="s">
         <v>10</v>
       </c>
@@ -3140,7 +2996,7 @@
       <c r="E37" s="38">
         <v>15</v>
       </c>
-      <c r="I37" s="96"/>
+      <c r="I37" s="77"/>
       <c r="J37" s="21" t="s">
         <v>10</v>
       </c>
@@ -3155,7 +3011,7 @@
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A38" s="93"/>
+      <c r="A38" s="74"/>
       <c r="B38" s="23" t="s">
         <v>12</v>
       </c>
@@ -3168,7 +3024,7 @@
       <c r="E38" s="38">
         <v>20</v>
       </c>
-      <c r="I38" s="96"/>
+      <c r="I38" s="77"/>
       <c r="J38" s="20" t="s">
         <v>12</v>
       </c>
@@ -3183,7 +3039,7 @@
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A39" s="93"/>
+      <c r="A39" s="74"/>
       <c r="B39" s="22" t="s">
         <v>14</v>
       </c>
@@ -3196,7 +3052,7 @@
       <c r="E39" s="38">
         <v>16</v>
       </c>
-      <c r="I39" s="96"/>
+      <c r="I39" s="77"/>
       <c r="J39" s="21" t="s">
         <v>14</v>
       </c>
@@ -3211,7 +3067,7 @@
       </c>
     </row>
     <row r="40" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="94"/>
+      <c r="A40" s="75"/>
       <c r="B40" s="41" t="s">
         <v>16</v>
       </c>
@@ -3224,7 +3080,7 @@
       <c r="E40" s="39">
         <v>16</v>
       </c>
-      <c r="I40" s="97"/>
+      <c r="I40" s="78"/>
       <c r="J40" s="28" t="s">
         <v>16</v>
       </c>
@@ -3239,7 +3095,7 @@
       </c>
     </row>
     <row r="41" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="92">
+      <c r="A41" s="73">
         <v>2025</v>
       </c>
       <c r="B41" s="40" t="s">
@@ -3254,7 +3110,7 @@
       <c r="E41" s="37">
         <v>14</v>
       </c>
-      <c r="I41" s="92">
+      <c r="I41" s="73">
         <v>2025</v>
       </c>
       <c r="J41" s="40" t="s">
@@ -3271,7 +3127,7 @@
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A42" s="93"/>
+      <c r="A42" s="74"/>
       <c r="B42" s="23" t="s">
         <v>8</v>
       </c>
@@ -3284,7 +3140,7 @@
       <c r="E42" s="38">
         <v>20</v>
       </c>
-      <c r="I42" s="93"/>
+      <c r="I42" s="74"/>
       <c r="J42" s="23" t="s">
         <v>8</v>
       </c>
@@ -3299,7 +3155,7 @@
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A43" s="93"/>
+      <c r="A43" s="74"/>
       <c r="B43" s="22" t="s">
         <v>10</v>
       </c>
@@ -3312,7 +3168,7 @@
       <c r="E43" s="38">
         <v>15</v>
       </c>
-      <c r="I43" s="93"/>
+      <c r="I43" s="74"/>
       <c r="J43" s="22" t="s">
         <v>10</v>
       </c>
@@ -3327,7 +3183,7 @@
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A44" s="93"/>
+      <c r="A44" s="74"/>
       <c r="B44" s="23" t="s">
         <v>12</v>
       </c>
@@ -3340,7 +3196,7 @@
       <c r="E44" s="38">
         <v>10</v>
       </c>
-      <c r="I44" s="93"/>
+      <c r="I44" s="74"/>
       <c r="J44" s="23" t="s">
         <v>12</v>
       </c>
@@ -3355,7 +3211,7 @@
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A45" s="93"/>
+      <c r="A45" s="74"/>
       <c r="B45" s="22" t="s">
         <v>14</v>
       </c>
@@ -3368,7 +3224,7 @@
       <c r="E45" s="38">
         <v>13</v>
       </c>
-      <c r="I45" s="93"/>
+      <c r="I45" s="74"/>
       <c r="J45" s="22" t="s">
         <v>14</v>
       </c>
@@ -3383,7 +3239,7 @@
       </c>
     </row>
     <row r="46" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="94"/>
+      <c r="A46" s="75"/>
       <c r="B46" s="41" t="s">
         <v>16</v>
       </c>
@@ -3396,7 +3252,7 @@
       <c r="E46" s="39">
         <v>16</v>
       </c>
-      <c r="I46" s="94"/>
+      <c r="I46" s="75"/>
       <c r="J46" s="41" t="s">
         <v>16</v>
       </c>
@@ -3410,142 +3266,325 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:13" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="48" spans="1:13" ht="31.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="47" t="s">
+    <row r="47" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="86">
+        <v>2026</v>
+      </c>
+      <c r="B47" s="40" t="s">
+        <v>6</v>
+      </c>
+      <c r="C47" s="26">
+        <v>10</v>
+      </c>
+      <c r="D47" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="E47" s="37">
+        <v>0</v>
+      </c>
+      <c r="I47" s="73">
+        <v>2026</v>
+      </c>
+      <c r="J47" s="40" t="s">
+        <v>6</v>
+      </c>
+      <c r="K47" s="26">
+        <v>2</v>
+      </c>
+      <c r="L47" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="M47" s="37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A48" s="83"/>
+      <c r="B48" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="C48" s="16">
+        <v>12</v>
+      </c>
+      <c r="D48" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="E48" s="38">
+        <v>0</v>
+      </c>
+      <c r="I48" s="74"/>
+      <c r="J48" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="K48" s="16">
         <v>3</v>
       </c>
-      <c r="B48" s="64" t="s">
+      <c r="L48" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="M48" s="38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A49" s="83"/>
+      <c r="B49" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C49" s="16">
         <v>18</v>
       </c>
-      <c r="I48" s="48" t="s">
+      <c r="D49" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E49" s="38">
+        <v>0</v>
+      </c>
+      <c r="I49" s="74"/>
+      <c r="J49" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="K49" s="16">
+        <v>1</v>
+      </c>
+      <c r="L49" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="M49" s="38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A50" s="83"/>
+      <c r="B50" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="C50" s="16">
+        <v>13</v>
+      </c>
+      <c r="D50" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="E50" s="38">
+        <v>0</v>
+      </c>
+      <c r="I50" s="74"/>
+      <c r="J50" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="K50" s="16">
+        <v>14</v>
+      </c>
+      <c r="L50" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="M50" s="38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A51" s="83"/>
+      <c r="B51" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="C51" s="16">
+        <v>11</v>
+      </c>
+      <c r="D51" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="E51" s="38">
+        <v>0</v>
+      </c>
+      <c r="I51" s="74"/>
+      <c r="J51" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="K51" s="16">
         <v>3</v>
       </c>
-      <c r="J48" s="63" t="s">
+      <c r="L51" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M51" s="38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="84"/>
+      <c r="B52" s="41" t="s">
+        <v>16</v>
+      </c>
+      <c r="C52" s="29">
+        <v>0</v>
+      </c>
+      <c r="D52" s="30" t="s">
+        <v>17</v>
+      </c>
+      <c r="E52" s="39">
+        <v>0</v>
+      </c>
+      <c r="I52" s="75"/>
+      <c r="J52" s="41" t="s">
+        <v>16</v>
+      </c>
+      <c r="K52" s="29">
+        <v>2</v>
+      </c>
+      <c r="L52" s="30" t="s">
+        <v>17</v>
+      </c>
+      <c r="M52" s="39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="54" spans="1:13" ht="31.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="94" t="s">
+        <v>3</v>
+      </c>
+      <c r="B54" s="99" t="s">
+        <v>18</v>
+      </c>
+      <c r="I54" s="97" t="s">
+        <v>3</v>
+      </c>
+      <c r="J54" s="98" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="82">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A55" s="93">
         <v>2019</v>
       </c>
-      <c r="B49" s="76">
+      <c r="B55" s="62">
         <v>143</v>
       </c>
-      <c r="I49" s="59">
+      <c r="I55" s="62">
         <v>2019</v>
       </c>
-      <c r="J49" s="49">
+      <c r="J55" s="62">
         <v>52</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A50" s="83">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A56" s="91">
         <v>2020</v>
       </c>
-      <c r="B50" s="44">
+      <c r="B56" s="8">
         <v>128</v>
       </c>
-      <c r="I50" s="60">
+      <c r="I56" s="8">
         <v>2020</v>
       </c>
-      <c r="J50" s="50">
+      <c r="J56" s="8">
         <v>32</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A51" s="84">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A57" s="91">
         <v>2021</v>
       </c>
-      <c r="B51" s="77">
+      <c r="B57" s="8">
         <v>139</v>
       </c>
-      <c r="I51" s="61">
+      <c r="I57" s="8">
         <v>2021</v>
       </c>
-      <c r="J51" s="51">
+      <c r="J57" s="8">
         <v>47</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A52" s="85">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A58" s="91">
         <v>2022</v>
       </c>
-      <c r="B52" s="78">
+      <c r="B58" s="8">
         <v>169</v>
       </c>
-      <c r="I52" s="62">
+      <c r="I58" s="8">
         <v>2022</v>
       </c>
-      <c r="J52" s="52">
+      <c r="J58" s="8">
         <v>30</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A53" s="86">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A59" s="91">
         <v>2023</v>
       </c>
-      <c r="B53" s="79">
+      <c r="B59" s="8">
         <v>144</v>
       </c>
-      <c r="I53" s="62">
+      <c r="I59" s="8">
         <v>2023</v>
       </c>
-      <c r="J53" s="52">
+      <c r="J59" s="8">
         <v>34</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A54" s="84">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A60" s="91">
         <v>2024</v>
       </c>
-      <c r="B54" s="80">
+      <c r="B60" s="8">
         <v>186</v>
       </c>
-      <c r="I54" s="62">
+      <c r="I60" s="8">
         <v>2024</v>
       </c>
-      <c r="J54" s="52">
+      <c r="J60" s="8">
         <v>25</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="84">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A61" s="91">
         <v>2025</v>
       </c>
-      <c r="B55" s="80">
+      <c r="B61" s="8">
         <v>190</v>
       </c>
-      <c r="I55" s="88">
+      <c r="I61" s="8">
         <v>2025</v>
       </c>
-      <c r="J55" s="53">
+      <c r="J61" s="8">
         <v>20</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="87" t="s">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A62" s="92">
+        <v>2026</v>
+      </c>
+      <c r="B62" s="8">
+        <v>64</v>
+      </c>
+      <c r="I62" s="96">
+        <v>2026</v>
+      </c>
+      <c r="J62" s="96">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A63" s="92" t="s">
         <v>20</v>
       </c>
-      <c r="B56" s="81">
-        <f>SUM(Table1[Total con querella])</f>
-        <v>1099</v>
-      </c>
-      <c r="I56" s="89" t="s">
+      <c r="B63" s="8">
+        <f>SUM(B55:B62)</f>
+        <v>1163</v>
+      </c>
+      <c r="I63" s="95" t="s">
         <v>20</v>
       </c>
-      <c r="J56" s="90">
-        <f>SUM(J49:J55)</f>
-        <v>240</v>
+      <c r="J63" s="95">
+        <f>SUM(J55:J62)</f>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="I11:I16"/>
-    <mergeCell ref="A41:A46"/>
-    <mergeCell ref="I41:I46"/>
-    <mergeCell ref="A35:A40"/>
-    <mergeCell ref="I35:I40"/>
+  <mergeCells count="19">
+    <mergeCell ref="A47:A52"/>
+    <mergeCell ref="I47:I52"/>
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="I3:M3"/>
@@ -3558,6 +3597,11 @@
     <mergeCell ref="A11:A16"/>
     <mergeCell ref="A5:A10"/>
     <mergeCell ref="I5:I10"/>
+    <mergeCell ref="I11:I16"/>
+    <mergeCell ref="A41:A46"/>
+    <mergeCell ref="I41:I46"/>
+    <mergeCell ref="A35:A40"/>
+    <mergeCell ref="I35:I40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">
@@ -3569,95 +3613,106 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:3" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="72" t="s">
+      <c r="B1" s="64" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="73" t="s">
+      <c r="C1" s="65" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="54">
+      <c r="A2" s="52">
         <v>2019</v>
       </c>
-      <c r="B2" s="49">
+      <c r="B2" s="47">
         <v>143</v>
       </c>
-      <c r="C2" s="49">
+      <c r="C2" s="47">
         <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="55">
+      <c r="A3" s="53">
         <v>2020</v>
       </c>
-      <c r="B3" s="50">
+      <c r="B3" s="48">
         <v>128</v>
       </c>
-      <c r="C3" s="50">
+      <c r="C3" s="48">
         <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="56">
+      <c r="A4" s="54">
         <v>2021</v>
       </c>
-      <c r="B4" s="51">
+      <c r="B4" s="49">
         <v>139</v>
       </c>
-      <c r="C4" s="51">
+      <c r="C4" s="49">
         <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="57">
+      <c r="A5" s="55">
         <v>2022</v>
       </c>
-      <c r="B5" s="52">
+      <c r="B5" s="50">
         <v>169</v>
       </c>
-      <c r="C5" s="52">
+      <c r="C5" s="50">
         <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="58">
+      <c r="A6" s="56">
         <v>2023</v>
       </c>
-      <c r="B6" s="53">
+      <c r="B6" s="51">
         <v>144</v>
       </c>
-      <c r="C6" s="52">
+      <c r="C6" s="50">
         <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="57">
+      <c r="A7" s="55">
         <v>2024</v>
       </c>
-      <c r="B7" s="75">
+      <c r="B7" s="67">
         <v>186</v>
       </c>
-      <c r="C7" s="52">
+      <c r="C7" s="50">
         <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="57">
+      <c r="A8" s="55">
         <v>2025</v>
       </c>
-      <c r="B8" s="75">
+      <c r="B8" s="67">
         <v>190</v>
       </c>
-      <c r="C8" s="52">
+      <c r="C8" s="50">
         <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="55">
+        <v>2026</v>
+      </c>
+      <c r="B9" s="67">
+        <v>75</v>
+      </c>
+      <c r="C9" s="50">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -3667,7 +3722,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -3676,16 +3731,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="74" t="s">
+      <c r="B1" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="74" t="s">
+      <c r="C1" s="66" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="74" t="s">
+      <c r="D1" s="66" t="s">
         <v>23</v>
       </c>
     </row>
@@ -3725,7 +3780,7 @@
         <v>53</v>
       </c>
       <c r="C4">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -3750,7 +3805,7 @@
         <v>2023</v>
       </c>
       <c r="B6">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C6">
         <v>77</v>
@@ -3767,7 +3822,7 @@
         <v>98</v>
       </c>
       <c r="C7">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -3781,9 +3836,23 @@
         <v>89</v>
       </c>
       <c r="C8">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>2026</v>
+      </c>
+      <c r="B9">
+        <v>31</v>
+      </c>
+      <c r="C9">
+        <v>44</v>
+      </c>
+      <c r="D9">
         <v>0</v>
       </c>
     </row>
@@ -3794,7 +3863,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5F89AC2-02D9-4754-B035-F9ADADF99A64}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.21875" customWidth="1"/>
@@ -3804,16 +3873,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="91" t="s">
+      <c r="A1" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="91" t="s">
+      <c r="B1" s="68" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="91" t="s">
+      <c r="C1" s="68" t="s">
         <v>25</v>
       </c>
-      <c r="D1" s="91" t="s">
+      <c r="D1" s="68" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3885,6 +3954,20 @@
       </c>
       <c r="D6">
         <v>181</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>2026</v>
+      </c>
+      <c r="B7">
+        <v>70</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3894,33 +3977,36 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3384D58-C6F0-4EC1-85A1-0F64609F10E6}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="91" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="68" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="91">
+      <c r="B1" s="68">
         <v>2021</v>
       </c>
-      <c r="C1" s="91">
+      <c r="C1" s="68">
         <v>2022</v>
       </c>
-      <c r="D1" s="91">
+      <c r="D1" s="68">
         <v>2023</v>
       </c>
-      <c r="E1" s="91">
+      <c r="E1" s="68">
         <v>2024</v>
       </c>
-      <c r="F1" s="91">
+      <c r="F1" s="68">
         <v>2025</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G1" s="68">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -3939,8 +4025,11 @@
       <c r="F2">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -3959,8 +4048,11 @@
       <c r="F3">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -3979,8 +4071,11 @@
       <c r="F4">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -3999,8 +4094,11 @@
       <c r="F5">
         <v>39</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G5">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>31</v>
       </c>
@@ -4019,8 +4117,11 @@
       <c r="F6">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -4039,8 +4140,11 @@
       <c r="F7">
         <v>17</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>33</v>
       </c>
@@ -4059,8 +4163,11 @@
       <c r="F8">
         <v>9</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>34</v>
       </c>
@@ -4079,8 +4186,11 @@
       <c r="F9">
         <v>5</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>35</v>
       </c>
@@ -4099,8 +4209,11 @@
       <c r="F10">
         <v>6</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -4119,8 +4232,11 @@
       <c r="F11">
         <v>6</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>36</v>
       </c>
@@ -4139,8 +4255,11 @@
       <c r="F12">
         <v>19</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -4159,8 +4278,11 @@
       <c r="F13">
         <v>44</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G13">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -4179,30 +4301,37 @@
       <c r="F14">
         <v>4</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="113" t="s">
+      <c r="G14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="69" t="s">
         <v>39</v>
       </c>
-      <c r="B15" s="113">
+      <c r="B15" s="69">
         <f t="shared" ref="B15:E15" si="0">SUM(B2:B14)</f>
         <v>141</v>
       </c>
-      <c r="C15" s="113">
+      <c r="C15" s="69">
         <f t="shared" si="0"/>
         <v>170</v>
       </c>
-      <c r="D15" s="113">
+      <c r="D15" s="69">
         <f t="shared" si="0"/>
         <v>145</v>
       </c>
-      <c r="E15" s="113">
+      <c r="E15" s="69">
         <f t="shared" si="0"/>
         <v>189</v>
       </c>
-      <c r="F15" s="113">
+      <c r="F15" s="69">
         <f>SUM(F2:F14)</f>
         <v>190</v>
+      </c>
+      <c r="G15" s="69">
+        <f>SUM(G2:G14)</f>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>